<commit_message>
Update gitignore and Selenium reports
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/excel/report.xlsx
+++ b/selenium-tests/reports/excel/report.xlsx
@@ -20,7 +20,7 @@
     <t>Report Generation Date:</t>
   </si>
   <si>
-    <t>11/6/2026, 1:42:47 pm</t>
+    <t>13/6/2026, 12:22:36 pm</t>
   </si>
   <si>
     <t>Target Environment:</t>
@@ -80,7 +80,7 @@
     <t>Total Run Duration</t>
   </si>
   <si>
-    <t>194.24 seconds</t>
+    <t>311.03 seconds</t>
   </si>
   <si>
     <t/>
@@ -1430,7 +1430,7 @@
         <v>35</v>
       </c>
       <c r="F2" s="12">
-        <v>3386</v>
+        <v>3964</v>
       </c>
       <c r="G2" s="13" t="s">
         <v>36</v>
@@ -1456,7 +1456,7 @@
         <v>35</v>
       </c>
       <c r="F3" s="12">
-        <v>1699</v>
+        <v>1942</v>
       </c>
       <c r="G3" s="13" t="s">
         <v>36</v>
@@ -1482,7 +1482,7 @@
         <v>35</v>
       </c>
       <c r="F4" s="12">
-        <v>388</v>
+        <v>683</v>
       </c>
       <c r="G4" s="13" t="s">
         <v>36</v>
@@ -1508,7 +1508,7 @@
         <v>35</v>
       </c>
       <c r="F5" s="12">
-        <v>3203</v>
+        <v>4919</v>
       </c>
       <c r="G5" s="13" t="s">
         <v>36</v>
@@ -1534,7 +1534,7 @@
         <v>35</v>
       </c>
       <c r="F6" s="12">
-        <v>1406</v>
+        <v>2448</v>
       </c>
       <c r="G6" s="13" t="s">
         <v>36</v>
@@ -1560,7 +1560,7 @@
         <v>35</v>
       </c>
       <c r="F7" s="12">
-        <v>2352</v>
+        <v>4412</v>
       </c>
       <c r="G7" s="13" t="s">
         <v>36</v>
@@ -1586,7 +1586,7 @@
         <v>35</v>
       </c>
       <c r="F8" s="12">
-        <v>2274</v>
+        <v>2625</v>
       </c>
       <c r="G8" s="13" t="s">
         <v>36</v>
@@ -1612,7 +1612,7 @@
         <v>35</v>
       </c>
       <c r="F9" s="12">
-        <v>1780</v>
+        <v>10184</v>
       </c>
       <c r="G9" s="13" t="s">
         <v>36</v>
@@ -1638,7 +1638,7 @@
         <v>35</v>
       </c>
       <c r="F10" s="12">
-        <v>4647</v>
+        <v>10209</v>
       </c>
       <c r="G10" s="13" t="s">
         <v>36</v>
@@ -1664,7 +1664,7 @@
         <v>35</v>
       </c>
       <c r="F11" s="12">
-        <v>788</v>
+        <v>10214</v>
       </c>
       <c r="G11" s="13" t="s">
         <v>36</v>
@@ -1690,7 +1690,7 @@
         <v>35</v>
       </c>
       <c r="F12" s="12">
-        <v>113</v>
+        <v>235</v>
       </c>
       <c r="G12" s="13" t="s">
         <v>36</v>
@@ -1716,7 +1716,7 @@
         <v>35</v>
       </c>
       <c r="F13" s="12">
-        <v>331</v>
+        <v>356</v>
       </c>
       <c r="G13" s="13" t="s">
         <v>36</v>
@@ -1742,7 +1742,7 @@
         <v>35</v>
       </c>
       <c r="F14" s="12">
-        <v>349</v>
+        <v>399</v>
       </c>
       <c r="G14" s="13" t="s">
         <v>36</v>
@@ -1768,7 +1768,7 @@
         <v>35</v>
       </c>
       <c r="F15" s="12">
-        <v>325</v>
+        <v>427</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>36</v>
@@ -1794,7 +1794,7 @@
         <v>35</v>
       </c>
       <c r="F16" s="12">
-        <v>201</v>
+        <v>372</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>36</v>
@@ -1820,7 +1820,7 @@
         <v>35</v>
       </c>
       <c r="F17" s="12">
-        <v>207</v>
+        <v>559</v>
       </c>
       <c r="G17" s="13" t="s">
         <v>36</v>
@@ -1846,7 +1846,7 @@
         <v>35</v>
       </c>
       <c r="F18" s="12">
-        <v>391</v>
+        <v>408</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>36</v>
@@ -1872,7 +1872,7 @@
         <v>35</v>
       </c>
       <c r="F19" s="12">
-        <v>138</v>
+        <v>279</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>36</v>
@@ -1898,7 +1898,7 @@
         <v>35</v>
       </c>
       <c r="F20" s="12">
-        <v>2238</v>
+        <v>1724</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>36</v>
@@ -1924,7 +1924,7 @@
         <v>35</v>
       </c>
       <c r="F21" s="12">
-        <v>263</v>
+        <v>1020</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>36</v>
@@ -1950,7 +1950,7 @@
         <v>35</v>
       </c>
       <c r="F22" s="12">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>36</v>
@@ -1976,7 +1976,7 @@
         <v>35</v>
       </c>
       <c r="F23" s="12">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>36</v>
@@ -2002,7 +2002,7 @@
         <v>35</v>
       </c>
       <c r="F24" s="12">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>36</v>
@@ -2028,7 +2028,7 @@
         <v>35</v>
       </c>
       <c r="F25" s="12">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>36</v>
@@ -2080,7 +2080,7 @@
         <v>35</v>
       </c>
       <c r="F27" s="12">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="G27" s="13" t="s">
         <v>36</v>
@@ -2106,7 +2106,7 @@
         <v>35</v>
       </c>
       <c r="F28" s="12">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="G28" s="13" t="s">
         <v>36</v>
@@ -2132,7 +2132,7 @@
         <v>35</v>
       </c>
       <c r="F29" s="12">
-        <v>3916</v>
+        <v>4396</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>36</v>
@@ -2158,7 +2158,7 @@
         <v>35</v>
       </c>
       <c r="F30" s="12">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="G30" s="13" t="s">
         <v>36</v>
@@ -2184,7 +2184,7 @@
         <v>35</v>
       </c>
       <c r="F31" s="12">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>36</v>
@@ -2210,7 +2210,7 @@
         <v>35</v>
       </c>
       <c r="F32" s="12">
-        <v>201</v>
+        <v>174</v>
       </c>
       <c r="G32" s="13" t="s">
         <v>36</v>
@@ -2236,7 +2236,7 @@
         <v>35</v>
       </c>
       <c r="F33" s="12">
-        <v>1200</v>
+        <v>1253</v>
       </c>
       <c r="G33" s="13" t="s">
         <v>36</v>
@@ -2262,7 +2262,7 @@
         <v>35</v>
       </c>
       <c r="F34" s="12">
-        <v>98</v>
+        <v>138</v>
       </c>
       <c r="G34" s="13" t="s">
         <v>36</v>
@@ -2288,7 +2288,7 @@
         <v>35</v>
       </c>
       <c r="F35" s="12">
-        <v>664</v>
+        <v>687</v>
       </c>
       <c r="G35" s="13" t="s">
         <v>36</v>
@@ -2314,7 +2314,7 @@
         <v>35</v>
       </c>
       <c r="F36" s="12">
-        <v>1168</v>
+        <v>1207</v>
       </c>
       <c r="G36" s="13" t="s">
         <v>36</v>
@@ -2340,7 +2340,7 @@
         <v>35</v>
       </c>
       <c r="F37" s="12">
-        <v>3128</v>
+        <v>3505</v>
       </c>
       <c r="G37" s="13" t="s">
         <v>36</v>
@@ -2366,7 +2366,7 @@
         <v>35</v>
       </c>
       <c r="F38" s="12">
-        <v>3505</v>
+        <v>3498</v>
       </c>
       <c r="G38" s="13" t="s">
         <v>36</v>
@@ -2392,7 +2392,7 @@
         <v>35</v>
       </c>
       <c r="F39" s="12">
-        <v>1157</v>
+        <v>1211</v>
       </c>
       <c r="G39" s="13" t="s">
         <v>36</v>
@@ -2418,7 +2418,7 @@
         <v>35</v>
       </c>
       <c r="F40" s="12">
-        <v>3094</v>
+        <v>3445</v>
       </c>
       <c r="G40" s="13" t="s">
         <v>36</v>
@@ -2444,7 +2444,7 @@
         <v>35</v>
       </c>
       <c r="F41" s="12">
-        <v>5116</v>
+        <v>4893</v>
       </c>
       <c r="G41" s="13" t="s">
         <v>36</v>
@@ -2470,7 +2470,7 @@
         <v>35</v>
       </c>
       <c r="F42" s="12">
-        <v>3580</v>
+        <v>3533</v>
       </c>
       <c r="G42" s="13" t="s">
         <v>36</v>
@@ -2496,7 +2496,7 @@
         <v>35</v>
       </c>
       <c r="F43" s="12">
-        <v>1315</v>
+        <v>1278</v>
       </c>
       <c r="G43" s="13" t="s">
         <v>36</v>
@@ -2522,7 +2522,7 @@
         <v>35</v>
       </c>
       <c r="F44" s="12">
-        <v>4678</v>
+        <v>4523</v>
       </c>
       <c r="G44" s="13" t="s">
         <v>36</v>
@@ -2548,7 +2548,7 @@
         <v>35</v>
       </c>
       <c r="F45" s="12">
-        <v>17651</v>
+        <v>17812</v>
       </c>
       <c r="G45" s="13" t="s">
         <v>36</v>
@@ -2574,7 +2574,7 @@
         <v>35</v>
       </c>
       <c r="F46" s="12">
-        <v>2568</v>
+        <v>2439</v>
       </c>
       <c r="G46" s="13" t="s">
         <v>36</v>
@@ -2600,7 +2600,7 @@
         <v>35</v>
       </c>
       <c r="F47" s="12">
-        <v>5797</v>
+        <v>6107</v>
       </c>
       <c r="G47" s="13" t="s">
         <v>36</v>
@@ -2626,7 +2626,7 @@
         <v>35</v>
       </c>
       <c r="F48" s="12">
-        <v>8105</v>
+        <v>8161</v>
       </c>
       <c r="G48" s="13" t="s">
         <v>36</v>
@@ -2652,7 +2652,7 @@
         <v>35</v>
       </c>
       <c r="F49" s="12">
-        <v>5056</v>
+        <v>5007</v>
       </c>
       <c r="G49" s="13" t="s">
         <v>36</v>
@@ -2678,7 +2678,7 @@
         <v>35</v>
       </c>
       <c r="F50" s="12">
-        <v>5126</v>
+        <v>5163</v>
       </c>
       <c r="G50" s="13" t="s">
         <v>36</v>
@@ -2704,7 +2704,7 @@
         <v>35</v>
       </c>
       <c r="F51" s="12">
-        <v>9836</v>
+        <v>10019</v>
       </c>
       <c r="G51" s="13" t="s">
         <v>36</v>
@@ -2730,7 +2730,7 @@
         <v>35</v>
       </c>
       <c r="F52" s="12">
-        <v>387</v>
+        <v>952</v>
       </c>
       <c r="G52" s="13" t="s">
         <v>36</v>
@@ -2756,7 +2756,7 @@
         <v>35</v>
       </c>
       <c r="F53" s="12">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="G53" s="13" t="s">
         <v>36</v>
@@ -2782,7 +2782,7 @@
         <v>35</v>
       </c>
       <c r="F54" s="12">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="G54" s="13" t="s">
         <v>36</v>
@@ -2808,7 +2808,7 @@
         <v>35</v>
       </c>
       <c r="F55" s="12">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="G55" s="13" t="s">
         <v>36</v>
@@ -2834,7 +2834,7 @@
         <v>35</v>
       </c>
       <c r="F56" s="12">
-        <v>1302</v>
+        <v>2047</v>
       </c>
       <c r="G56" s="13" t="s">
         <v>36</v>
@@ -2860,7 +2860,7 @@
         <v>35</v>
       </c>
       <c r="F57" s="12">
-        <v>1130</v>
+        <v>1228</v>
       </c>
       <c r="G57" s="13" t="s">
         <v>36</v>
@@ -2886,7 +2886,7 @@
         <v>35</v>
       </c>
       <c r="F58" s="12">
-        <v>1114</v>
+        <v>1191</v>
       </c>
       <c r="G58" s="13" t="s">
         <v>36</v>
@@ -2912,7 +2912,7 @@
         <v>35</v>
       </c>
       <c r="F59" s="12">
-        <v>1190</v>
+        <v>1199</v>
       </c>
       <c r="G59" s="13" t="s">
         <v>36</v>
@@ -2938,7 +2938,7 @@
         <v>35</v>
       </c>
       <c r="F60" s="12">
-        <v>385</v>
+        <v>750</v>
       </c>
       <c r="G60" s="13" t="s">
         <v>36</v>
@@ -2964,7 +2964,7 @@
         <v>35</v>
       </c>
       <c r="F61" s="12">
-        <v>1714</v>
+        <v>2190</v>
       </c>
       <c r="G61" s="13" t="s">
         <v>36</v>
@@ -2990,7 +2990,7 @@
         <v>35</v>
       </c>
       <c r="F62" s="12">
-        <v>1595</v>
+        <v>1594</v>
       </c>
       <c r="G62" s="13" t="s">
         <v>36</v>
@@ -3016,7 +3016,7 @@
         <v>35</v>
       </c>
       <c r="F63" s="12">
-        <v>1119</v>
+        <v>1596</v>
       </c>
       <c r="G63" s="13" t="s">
         <v>36</v>
@@ -3042,7 +3042,7 @@
         <v>35</v>
       </c>
       <c r="F64" s="12">
-        <v>139</v>
+        <v>596</v>
       </c>
       <c r="G64" s="13" t="s">
         <v>36</v>
@@ -3068,7 +3068,7 @@
         <v>35</v>
       </c>
       <c r="F65" s="12">
-        <v>549</v>
+        <v>466</v>
       </c>
       <c r="G65" s="13" t="s">
         <v>36</v>
@@ -3094,7 +3094,7 @@
         <v>35</v>
       </c>
       <c r="F66" s="12">
-        <v>82</v>
+        <v>520</v>
       </c>
       <c r="G66" s="13" t="s">
         <v>36</v>
@@ -3120,7 +3120,7 @@
         <v>35</v>
       </c>
       <c r="F67" s="12">
-        <v>290</v>
+        <v>96</v>
       </c>
       <c r="G67" s="13" t="s">
         <v>36</v>
@@ -3146,7 +3146,7 @@
         <v>35</v>
       </c>
       <c r="F68" s="12">
-        <v>1138</v>
+        <v>1214</v>
       </c>
       <c r="G68" s="13" t="s">
         <v>36</v>
@@ -3172,7 +3172,7 @@
         <v>35</v>
       </c>
       <c r="F69" s="12">
-        <v>1304</v>
+        <v>1740</v>
       </c>
       <c r="G69" s="13" t="s">
         <v>36</v>
@@ -3198,7 +3198,7 @@
         <v>35</v>
       </c>
       <c r="F70" s="12">
-        <v>2055</v>
+        <v>2096</v>
       </c>
       <c r="G70" s="13" t="s">
         <v>36</v>
@@ -3224,7 +3224,7 @@
         <v>35</v>
       </c>
       <c r="F71" s="12">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G71" s="13" t="s">
         <v>36</v>
@@ -3250,7 +3250,7 @@
         <v>35</v>
       </c>
       <c r="F72" s="12">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="G72" s="13" t="s">
         <v>36</v>
@@ -3276,7 +3276,7 @@
         <v>35</v>
       </c>
       <c r="F73" s="12">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="G73" s="13" t="s">
         <v>36</v>
@@ -3302,7 +3302,7 @@
         <v>35</v>
       </c>
       <c r="F74" s="12">
-        <v>357</v>
+        <v>282</v>
       </c>
       <c r="G74" s="13" t="s">
         <v>36</v>
@@ -3328,7 +3328,7 @@
         <v>35</v>
       </c>
       <c r="F75" s="12">
-        <v>904</v>
+        <v>797</v>
       </c>
       <c r="G75" s="13" t="s">
         <v>36</v>
@@ -3354,7 +3354,7 @@
         <v>35</v>
       </c>
       <c r="F76" s="12">
-        <v>928</v>
+        <v>855</v>
       </c>
       <c r="G76" s="13" t="s">
         <v>36</v>
@@ -3406,7 +3406,7 @@
         <v>35</v>
       </c>
       <c r="F78" s="12">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="G78" s="13" t="s">
         <v>36</v>
@@ -3432,7 +3432,7 @@
         <v>35</v>
       </c>
       <c r="F79" s="12">
-        <v>946</v>
+        <v>805</v>
       </c>
       <c r="G79" s="13" t="s">
         <v>36</v>
@@ -3458,7 +3458,7 @@
         <v>35</v>
       </c>
       <c r="F80" s="12">
-        <v>472</v>
+        <v>151</v>
       </c>
       <c r="G80" s="13" t="s">
         <v>36</v>
@@ -3484,7 +3484,7 @@
         <v>35</v>
       </c>
       <c r="F81" s="12">
-        <v>191</v>
+        <v>10155</v>
       </c>
       <c r="G81" s="13" t="s">
         <v>36</v>
@@ -3510,7 +3510,7 @@
         <v>35</v>
       </c>
       <c r="F82" s="12">
-        <v>2116</v>
+        <v>10706</v>
       </c>
       <c r="G82" s="13" t="s">
         <v>36</v>
@@ -3536,7 +3536,7 @@
         <v>35</v>
       </c>
       <c r="F83" s="12">
-        <v>475</v>
+        <v>10165</v>
       </c>
       <c r="G83" s="13" t="s">
         <v>36</v>
@@ -3562,7 +3562,7 @@
         <v>35</v>
       </c>
       <c r="F84" s="12">
-        <v>7225</v>
+        <v>10574</v>
       </c>
       <c r="G84" s="13" t="s">
         <v>36</v>
@@ -3588,7 +3588,7 @@
         <v>35</v>
       </c>
       <c r="F85" s="12">
-        <v>1508</v>
+        <v>16845</v>
       </c>
       <c r="G85" s="13" t="s">
         <v>36</v>
@@ -3614,7 +3614,7 @@
         <v>35</v>
       </c>
       <c r="F86" s="12">
-        <v>8768</v>
+        <v>10565</v>
       </c>
       <c r="G86" s="13" t="s">
         <v>36</v>
@@ -3640,7 +3640,7 @@
         <v>35</v>
       </c>
       <c r="F87" s="12">
-        <v>2117</v>
+        <v>10040</v>
       </c>
       <c r="G87" s="13" t="s">
         <v>36</v>
@@ -3666,7 +3666,7 @@
         <v>35</v>
       </c>
       <c r="F88" s="12">
-        <v>5125</v>
+        <v>16060</v>
       </c>
       <c r="G88" s="13" t="s">
         <v>36</v>
@@ -3692,7 +3692,7 @@
         <v>35</v>
       </c>
       <c r="F89" s="12">
-        <v>292</v>
+        <v>392</v>
       </c>
       <c r="G89" s="13" t="s">
         <v>36</v>
@@ -3718,7 +3718,7 @@
         <v>35</v>
       </c>
       <c r="F90" s="12">
-        <v>2615</v>
+        <v>2732</v>
       </c>
       <c r="G90" s="13" t="s">
         <v>36</v>
@@ -3744,7 +3744,7 @@
         <v>35</v>
       </c>
       <c r="F91" s="12">
-        <v>2551</v>
+        <v>2785</v>
       </c>
       <c r="G91" s="13" t="s">
         <v>36</v>
@@ -3770,7 +3770,7 @@
         <v>35</v>
       </c>
       <c r="F92" s="12">
-        <v>1506</v>
+        <v>1519</v>
       </c>
       <c r="G92" s="13" t="s">
         <v>36</v>
@@ -3796,7 +3796,7 @@
         <v>35</v>
       </c>
       <c r="F93" s="12">
-        <v>1323</v>
+        <v>1626</v>
       </c>
       <c r="G93" s="13" t="s">
         <v>36</v>
@@ -3822,7 +3822,7 @@
         <v>35</v>
       </c>
       <c r="F94" s="12">
-        <v>843</v>
+        <v>1229</v>
       </c>
       <c r="G94" s="13" t="s">
         <v>36</v>
@@ -3848,7 +3848,7 @@
         <v>35</v>
       </c>
       <c r="F95" s="12">
-        <v>214</v>
+        <v>185</v>
       </c>
       <c r="G95" s="13" t="s">
         <v>36</v>
@@ -3874,7 +3874,7 @@
         <v>35</v>
       </c>
       <c r="F96" s="12">
-        <v>793</v>
+        <v>906</v>
       </c>
       <c r="G96" s="13" t="s">
         <v>36</v>
@@ -3900,7 +3900,7 @@
         <v>35</v>
       </c>
       <c r="F97" s="12">
-        <v>1237</v>
+        <v>2195</v>
       </c>
       <c r="G97" s="13" t="s">
         <v>36</v>
@@ -3926,7 +3926,7 @@
         <v>35</v>
       </c>
       <c r="F98" s="12">
-        <v>3793</v>
+        <v>6047</v>
       </c>
       <c r="G98" s="13" t="s">
         <v>36</v>
@@ -3952,7 +3952,7 @@
         <v>35</v>
       </c>
       <c r="F99" s="12">
-        <v>6547</v>
+        <v>8282</v>
       </c>
       <c r="G99" s="13" t="s">
         <v>36</v>
@@ -3978,7 +3978,7 @@
         <v>35</v>
       </c>
       <c r="F100" s="12">
-        <v>2977</v>
+        <v>3287</v>
       </c>
       <c r="G100" s="13" t="s">
         <v>36</v>
@@ -4004,7 +4004,7 @@
         <v>35</v>
       </c>
       <c r="F101" s="12">
-        <v>4263</v>
+        <v>8646</v>
       </c>
       <c r="G101" s="13" t="s">
         <v>36</v>
@@ -4030,7 +4030,7 @@
         <v>35</v>
       </c>
       <c r="F102" s="12">
-        <v>410</v>
+        <v>2064</v>
       </c>
       <c r="G102" s="13" t="s">
         <v>36</v>
@@ -4056,7 +4056,7 @@
         <v>35</v>
       </c>
       <c r="F103" s="12">
-        <v>157</v>
+        <v>254</v>
       </c>
       <c r="G103" s="13" t="s">
         <v>36</v>
@@ -4082,7 +4082,7 @@
         <v>35</v>
       </c>
       <c r="F104" s="12">
-        <v>483</v>
+        <v>1042</v>
       </c>
       <c r="G104" s="13" t="s">
         <v>36</v>
@@ -4108,7 +4108,7 @@
         <v>35</v>
       </c>
       <c r="F105" s="12">
-        <v>3427</v>
+        <v>3775</v>
       </c>
       <c r="G105" s="13" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
Improve web app UI and fixes
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/excel/report.xlsx
+++ b/selenium-tests/reports/excel/report.xlsx
@@ -20,7 +20,7 @@
     <t>Report Generation Date:</t>
   </si>
   <si>
-    <t>13/6/2026, 12:22:36 pm</t>
+    <t>14/6/2026, 12:58:02 pm</t>
   </si>
   <si>
     <t>Target Environment:</t>
@@ -80,7 +80,7 @@
     <t>Total Run Duration</t>
   </si>
   <si>
-    <t>311.03 seconds</t>
+    <t>273.60 seconds</t>
   </si>
   <si>
     <t/>
@@ -1430,7 +1430,7 @@
         <v>35</v>
       </c>
       <c r="F2" s="12">
-        <v>3964</v>
+        <v>3627</v>
       </c>
       <c r="G2" s="13" t="s">
         <v>36</v>
@@ -1456,7 +1456,7 @@
         <v>35</v>
       </c>
       <c r="F3" s="12">
-        <v>1942</v>
+        <v>1969</v>
       </c>
       <c r="G3" s="13" t="s">
         <v>36</v>
@@ -1482,7 +1482,7 @@
         <v>35</v>
       </c>
       <c r="F4" s="12">
-        <v>683</v>
+        <v>390</v>
       </c>
       <c r="G4" s="13" t="s">
         <v>36</v>
@@ -1508,7 +1508,7 @@
         <v>35</v>
       </c>
       <c r="F5" s="12">
-        <v>4919</v>
+        <v>2940</v>
       </c>
       <c r="G5" s="13" t="s">
         <v>36</v>
@@ -1534,7 +1534,7 @@
         <v>35</v>
       </c>
       <c r="F6" s="12">
-        <v>2448</v>
+        <v>1468</v>
       </c>
       <c r="G6" s="13" t="s">
         <v>36</v>
@@ -1560,7 +1560,7 @@
         <v>35</v>
       </c>
       <c r="F7" s="12">
-        <v>4412</v>
+        <v>2010</v>
       </c>
       <c r="G7" s="13" t="s">
         <v>36</v>
@@ -1586,7 +1586,7 @@
         <v>35</v>
       </c>
       <c r="F8" s="12">
-        <v>2625</v>
+        <v>2194</v>
       </c>
       <c r="G8" s="13" t="s">
         <v>36</v>
@@ -1612,7 +1612,7 @@
         <v>35</v>
       </c>
       <c r="F9" s="12">
-        <v>10184</v>
+        <v>1582</v>
       </c>
       <c r="G9" s="13" t="s">
         <v>36</v>
@@ -1638,7 +1638,7 @@
         <v>35</v>
       </c>
       <c r="F10" s="12">
-        <v>10209</v>
+        <v>3765</v>
       </c>
       <c r="G10" s="13" t="s">
         <v>36</v>
@@ -1664,7 +1664,7 @@
         <v>35</v>
       </c>
       <c r="F11" s="12">
-        <v>10214</v>
+        <v>759</v>
       </c>
       <c r="G11" s="13" t="s">
         <v>36</v>
@@ -1690,7 +1690,7 @@
         <v>35</v>
       </c>
       <c r="F12" s="12">
-        <v>235</v>
+        <v>97</v>
       </c>
       <c r="G12" s="13" t="s">
         <v>36</v>
@@ -1716,7 +1716,7 @@
         <v>35</v>
       </c>
       <c r="F13" s="12">
-        <v>356</v>
+        <v>101</v>
       </c>
       <c r="G13" s="13" t="s">
         <v>36</v>
@@ -1742,7 +1742,7 @@
         <v>35</v>
       </c>
       <c r="F14" s="12">
-        <v>399</v>
+        <v>244</v>
       </c>
       <c r="G14" s="13" t="s">
         <v>36</v>
@@ -1768,7 +1768,7 @@
         <v>35</v>
       </c>
       <c r="F15" s="12">
-        <v>427</v>
+        <v>190</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>36</v>
@@ -1794,7 +1794,7 @@
         <v>35</v>
       </c>
       <c r="F16" s="12">
-        <v>372</v>
+        <v>178</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>36</v>
@@ -1820,7 +1820,7 @@
         <v>35</v>
       </c>
       <c r="F17" s="12">
-        <v>559</v>
+        <v>170</v>
       </c>
       <c r="G17" s="13" t="s">
         <v>36</v>
@@ -1846,7 +1846,7 @@
         <v>35</v>
       </c>
       <c r="F18" s="12">
-        <v>408</v>
+        <v>185</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>36</v>
@@ -1872,7 +1872,7 @@
         <v>35</v>
       </c>
       <c r="F19" s="12">
-        <v>279</v>
+        <v>151</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>36</v>
@@ -1898,7 +1898,7 @@
         <v>35</v>
       </c>
       <c r="F20" s="12">
-        <v>1724</v>
+        <v>983</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>36</v>
@@ -1924,7 +1924,7 @@
         <v>35</v>
       </c>
       <c r="F21" s="12">
-        <v>1020</v>
+        <v>207</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>36</v>
@@ -1950,7 +1950,7 @@
         <v>35</v>
       </c>
       <c r="F22" s="12">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>36</v>
@@ -1976,7 +1976,7 @@
         <v>35</v>
       </c>
       <c r="F23" s="12">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>36</v>
@@ -2002,7 +2002,7 @@
         <v>35</v>
       </c>
       <c r="F24" s="12">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>36</v>
@@ -2028,7 +2028,7 @@
         <v>35</v>
       </c>
       <c r="F25" s="12">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>36</v>
@@ -2054,7 +2054,7 @@
         <v>35</v>
       </c>
       <c r="F26" s="12">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G26" s="13" t="s">
         <v>36</v>
@@ -2080,7 +2080,7 @@
         <v>35</v>
       </c>
       <c r="F27" s="12">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G27" s="13" t="s">
         <v>36</v>
@@ -2106,7 +2106,7 @@
         <v>35</v>
       </c>
       <c r="F28" s="12">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="G28" s="13" t="s">
         <v>36</v>
@@ -2132,7 +2132,7 @@
         <v>35</v>
       </c>
       <c r="F29" s="12">
-        <v>4396</v>
+        <v>3712</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>36</v>
@@ -2158,7 +2158,7 @@
         <v>35</v>
       </c>
       <c r="F30" s="12">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G30" s="13" t="s">
         <v>36</v>
@@ -2184,7 +2184,7 @@
         <v>35</v>
       </c>
       <c r="F31" s="12">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>36</v>
@@ -2210,7 +2210,7 @@
         <v>35</v>
       </c>
       <c r="F32" s="12">
-        <v>174</v>
+        <v>241</v>
       </c>
       <c r="G32" s="13" t="s">
         <v>36</v>
@@ -2236,7 +2236,7 @@
         <v>35</v>
       </c>
       <c r="F33" s="12">
-        <v>1253</v>
+        <v>1126</v>
       </c>
       <c r="G33" s="13" t="s">
         <v>36</v>
@@ -2262,7 +2262,7 @@
         <v>35</v>
       </c>
       <c r="F34" s="12">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="G34" s="13" t="s">
         <v>36</v>
@@ -2288,7 +2288,7 @@
         <v>35</v>
       </c>
       <c r="F35" s="12">
-        <v>687</v>
+        <v>653</v>
       </c>
       <c r="G35" s="13" t="s">
         <v>36</v>
@@ -2314,7 +2314,7 @@
         <v>35</v>
       </c>
       <c r="F36" s="12">
-        <v>1207</v>
+        <v>1149</v>
       </c>
       <c r="G36" s="13" t="s">
         <v>36</v>
@@ -2340,7 +2340,7 @@
         <v>35</v>
       </c>
       <c r="F37" s="12">
-        <v>3505</v>
+        <v>2682</v>
       </c>
       <c r="G37" s="13" t="s">
         <v>36</v>
@@ -2366,7 +2366,7 @@
         <v>35</v>
       </c>
       <c r="F38" s="12">
-        <v>3498</v>
+        <v>3246</v>
       </c>
       <c r="G38" s="13" t="s">
         <v>36</v>
@@ -2392,7 +2392,7 @@
         <v>35</v>
       </c>
       <c r="F39" s="12">
-        <v>1211</v>
+        <v>1109</v>
       </c>
       <c r="G39" s="13" t="s">
         <v>36</v>
@@ -2418,7 +2418,7 @@
         <v>35</v>
       </c>
       <c r="F40" s="12">
-        <v>3445</v>
+        <v>2600</v>
       </c>
       <c r="G40" s="13" t="s">
         <v>36</v>
@@ -2444,7 +2444,7 @@
         <v>35</v>
       </c>
       <c r="F41" s="12">
-        <v>4893</v>
+        <v>4438</v>
       </c>
       <c r="G41" s="13" t="s">
         <v>36</v>
@@ -2470,7 +2470,7 @@
         <v>35</v>
       </c>
       <c r="F42" s="12">
-        <v>3533</v>
+        <v>3194</v>
       </c>
       <c r="G42" s="13" t="s">
         <v>36</v>
@@ -2496,7 +2496,7 @@
         <v>35</v>
       </c>
       <c r="F43" s="12">
-        <v>1278</v>
+        <v>1013</v>
       </c>
       <c r="G43" s="13" t="s">
         <v>36</v>
@@ -2522,7 +2522,7 @@
         <v>35</v>
       </c>
       <c r="F44" s="12">
-        <v>4523</v>
+        <v>4040</v>
       </c>
       <c r="G44" s="13" t="s">
         <v>36</v>
@@ -2548,7 +2548,7 @@
         <v>35</v>
       </c>
       <c r="F45" s="12">
-        <v>17812</v>
+        <v>17383</v>
       </c>
       <c r="G45" s="13" t="s">
         <v>36</v>
@@ -2574,7 +2574,7 @@
         <v>35</v>
       </c>
       <c r="F46" s="12">
-        <v>2439</v>
+        <v>2270</v>
       </c>
       <c r="G46" s="13" t="s">
         <v>36</v>
@@ -2600,7 +2600,7 @@
         <v>35</v>
       </c>
       <c r="F47" s="12">
-        <v>6107</v>
+        <v>5416</v>
       </c>
       <c r="G47" s="13" t="s">
         <v>36</v>
@@ -2626,7 +2626,7 @@
         <v>35</v>
       </c>
       <c r="F48" s="12">
-        <v>8161</v>
+        <v>8064</v>
       </c>
       <c r="G48" s="13" t="s">
         <v>36</v>
@@ -2652,7 +2652,7 @@
         <v>35</v>
       </c>
       <c r="F49" s="12">
-        <v>5007</v>
+        <v>4318</v>
       </c>
       <c r="G49" s="13" t="s">
         <v>36</v>
@@ -2678,7 +2678,7 @@
         <v>35</v>
       </c>
       <c r="F50" s="12">
-        <v>5163</v>
+        <v>5122</v>
       </c>
       <c r="G50" s="13" t="s">
         <v>36</v>
@@ -2704,7 +2704,7 @@
         <v>35</v>
       </c>
       <c r="F51" s="12">
-        <v>10019</v>
+        <v>9581</v>
       </c>
       <c r="G51" s="13" t="s">
         <v>36</v>
@@ -2730,7 +2730,7 @@
         <v>35</v>
       </c>
       <c r="F52" s="12">
-        <v>952</v>
+        <v>360</v>
       </c>
       <c r="G52" s="13" t="s">
         <v>36</v>
@@ -2756,7 +2756,7 @@
         <v>35</v>
       </c>
       <c r="F53" s="12">
-        <v>85</v>
+        <v>44</v>
       </c>
       <c r="G53" s="13" t="s">
         <v>36</v>
@@ -2782,7 +2782,7 @@
         <v>35</v>
       </c>
       <c r="F54" s="12">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="G54" s="13" t="s">
         <v>36</v>
@@ -2808,7 +2808,7 @@
         <v>35</v>
       </c>
       <c r="F55" s="12">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G55" s="13" t="s">
         <v>36</v>
@@ -2834,7 +2834,7 @@
         <v>35</v>
       </c>
       <c r="F56" s="12">
-        <v>2047</v>
+        <v>1494</v>
       </c>
       <c r="G56" s="13" t="s">
         <v>36</v>
@@ -2860,7 +2860,7 @@
         <v>35</v>
       </c>
       <c r="F57" s="12">
-        <v>1228</v>
+        <v>1117</v>
       </c>
       <c r="G57" s="13" t="s">
         <v>36</v>
@@ -2886,7 +2886,7 @@
         <v>35</v>
       </c>
       <c r="F58" s="12">
-        <v>1191</v>
+        <v>1185</v>
       </c>
       <c r="G58" s="13" t="s">
         <v>36</v>
@@ -2912,7 +2912,7 @@
         <v>35</v>
       </c>
       <c r="F59" s="12">
-        <v>1199</v>
+        <v>1120</v>
       </c>
       <c r="G59" s="13" t="s">
         <v>36</v>
@@ -2938,7 +2938,7 @@
         <v>35</v>
       </c>
       <c r="F60" s="12">
-        <v>750</v>
+        <v>490</v>
       </c>
       <c r="G60" s="13" t="s">
         <v>36</v>
@@ -2964,7 +2964,7 @@
         <v>35</v>
       </c>
       <c r="F61" s="12">
-        <v>2190</v>
+        <v>1575</v>
       </c>
       <c r="G61" s="13" t="s">
         <v>36</v>
@@ -2990,7 +2990,7 @@
         <v>35</v>
       </c>
       <c r="F62" s="12">
-        <v>1594</v>
+        <v>1591</v>
       </c>
       <c r="G62" s="13" t="s">
         <v>36</v>
@@ -3016,7 +3016,7 @@
         <v>35</v>
       </c>
       <c r="F63" s="12">
-        <v>1596</v>
+        <v>878</v>
       </c>
       <c r="G63" s="13" t="s">
         <v>36</v>
@@ -3042,7 +3042,7 @@
         <v>35</v>
       </c>
       <c r="F64" s="12">
-        <v>596</v>
+        <v>493</v>
       </c>
       <c r="G64" s="13" t="s">
         <v>36</v>
@@ -3068,7 +3068,7 @@
         <v>35</v>
       </c>
       <c r="F65" s="12">
-        <v>466</v>
+        <v>337</v>
       </c>
       <c r="G65" s="13" t="s">
         <v>36</v>
@@ -3094,7 +3094,7 @@
         <v>35</v>
       </c>
       <c r="F66" s="12">
-        <v>520</v>
+        <v>534</v>
       </c>
       <c r="G66" s="13" t="s">
         <v>36</v>
@@ -3120,7 +3120,7 @@
         <v>35</v>
       </c>
       <c r="F67" s="12">
-        <v>96</v>
+        <v>254</v>
       </c>
       <c r="G67" s="13" t="s">
         <v>36</v>
@@ -3146,7 +3146,7 @@
         <v>35</v>
       </c>
       <c r="F68" s="12">
-        <v>1214</v>
+        <v>1114</v>
       </c>
       <c r="G68" s="13" t="s">
         <v>36</v>
@@ -3172,7 +3172,7 @@
         <v>35</v>
       </c>
       <c r="F69" s="12">
-        <v>1740</v>
+        <v>10814</v>
       </c>
       <c r="G69" s="13" t="s">
         <v>36</v>
@@ -3198,7 +3198,7 @@
         <v>35</v>
       </c>
       <c r="F70" s="12">
-        <v>2096</v>
+        <v>17212</v>
       </c>
       <c r="G70" s="13" t="s">
         <v>36</v>
@@ -3224,7 +3224,7 @@
         <v>35</v>
       </c>
       <c r="F71" s="12">
-        <v>59</v>
+        <v>10036</v>
       </c>
       <c r="G71" s="13" t="s">
         <v>36</v>
@@ -3250,7 +3250,7 @@
         <v>35</v>
       </c>
       <c r="F72" s="12">
-        <v>84</v>
+        <v>10027</v>
       </c>
       <c r="G72" s="13" t="s">
         <v>36</v>
@@ -3276,7 +3276,7 @@
         <v>35</v>
       </c>
       <c r="F73" s="12">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="G73" s="13" t="s">
         <v>36</v>
@@ -3302,7 +3302,7 @@
         <v>35</v>
       </c>
       <c r="F74" s="12">
-        <v>282</v>
+        <v>10137</v>
       </c>
       <c r="G74" s="13" t="s">
         <v>36</v>
@@ -3328,7 +3328,7 @@
         <v>35</v>
       </c>
       <c r="F75" s="12">
-        <v>797</v>
+        <v>10034</v>
       </c>
       <c r="G75" s="13" t="s">
         <v>36</v>
@@ -3354,7 +3354,7 @@
         <v>35</v>
       </c>
       <c r="F76" s="12">
-        <v>855</v>
+        <v>10011</v>
       </c>
       <c r="G76" s="13" t="s">
         <v>36</v>
@@ -3380,7 +3380,7 @@
         <v>35</v>
       </c>
       <c r="F77" s="12">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="G77" s="13" t="s">
         <v>36</v>
@@ -3406,7 +3406,7 @@
         <v>35</v>
       </c>
       <c r="F78" s="12">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="G78" s="13" t="s">
         <v>36</v>
@@ -3432,7 +3432,7 @@
         <v>35</v>
       </c>
       <c r="F79" s="12">
-        <v>805</v>
+        <v>10028</v>
       </c>
       <c r="G79" s="13" t="s">
         <v>36</v>
@@ -3458,7 +3458,7 @@
         <v>35</v>
       </c>
       <c r="F80" s="12">
-        <v>151</v>
+        <v>7</v>
       </c>
       <c r="G80" s="13" t="s">
         <v>36</v>
@@ -3484,7 +3484,7 @@
         <v>35</v>
       </c>
       <c r="F81" s="12">
-        <v>10155</v>
+        <v>151</v>
       </c>
       <c r="G81" s="13" t="s">
         <v>36</v>
@@ -3510,7 +3510,7 @@
         <v>35</v>
       </c>
       <c r="F82" s="12">
-        <v>10706</v>
+        <v>2182</v>
       </c>
       <c r="G82" s="13" t="s">
         <v>36</v>
@@ -3536,7 +3536,7 @@
         <v>35</v>
       </c>
       <c r="F83" s="12">
-        <v>10165</v>
+        <v>487</v>
       </c>
       <c r="G83" s="13" t="s">
         <v>36</v>
@@ -3562,7 +3562,7 @@
         <v>35</v>
       </c>
       <c r="F84" s="12">
-        <v>10574</v>
+        <v>6687</v>
       </c>
       <c r="G84" s="13" t="s">
         <v>36</v>
@@ -3588,7 +3588,7 @@
         <v>35</v>
       </c>
       <c r="F85" s="12">
-        <v>16845</v>
+        <v>1509</v>
       </c>
       <c r="G85" s="13" t="s">
         <v>36</v>
@@ -3614,7 +3614,7 @@
         <v>35</v>
       </c>
       <c r="F86" s="12">
-        <v>10565</v>
+        <v>8103</v>
       </c>
       <c r="G86" s="13" t="s">
         <v>36</v>
@@ -3640,7 +3640,7 @@
         <v>35</v>
       </c>
       <c r="F87" s="12">
-        <v>10040</v>
+        <v>2113</v>
       </c>
       <c r="G87" s="13" t="s">
         <v>36</v>
@@ -3666,7 +3666,7 @@
         <v>35</v>
       </c>
       <c r="F88" s="12">
-        <v>16060</v>
+        <v>5129</v>
       </c>
       <c r="G88" s="13" t="s">
         <v>36</v>
@@ -3692,7 +3692,7 @@
         <v>35</v>
       </c>
       <c r="F89" s="12">
-        <v>392</v>
+        <v>303</v>
       </c>
       <c r="G89" s="13" t="s">
         <v>36</v>
@@ -3718,7 +3718,7 @@
         <v>35</v>
       </c>
       <c r="F90" s="12">
-        <v>2732</v>
+        <v>2604</v>
       </c>
       <c r="G90" s="13" t="s">
         <v>36</v>
@@ -3744,7 +3744,7 @@
         <v>35</v>
       </c>
       <c r="F91" s="12">
-        <v>2785</v>
+        <v>2453</v>
       </c>
       <c r="G91" s="13" t="s">
         <v>36</v>
@@ -3770,7 +3770,7 @@
         <v>35</v>
       </c>
       <c r="F92" s="12">
-        <v>1519</v>
+        <v>1515</v>
       </c>
       <c r="G92" s="13" t="s">
         <v>36</v>
@@ -3796,7 +3796,7 @@
         <v>35</v>
       </c>
       <c r="F93" s="12">
-        <v>1626</v>
+        <v>1302</v>
       </c>
       <c r="G93" s="13" t="s">
         <v>36</v>
@@ -3822,7 +3822,7 @@
         <v>35</v>
       </c>
       <c r="F94" s="12">
-        <v>1229</v>
+        <v>829</v>
       </c>
       <c r="G94" s="13" t="s">
         <v>36</v>
@@ -3848,7 +3848,7 @@
         <v>35</v>
       </c>
       <c r="F95" s="12">
-        <v>185</v>
+        <v>10054</v>
       </c>
       <c r="G95" s="13" t="s">
         <v>36</v>
@@ -3874,7 +3874,7 @@
         <v>35</v>
       </c>
       <c r="F96" s="12">
-        <v>906</v>
+        <v>54</v>
       </c>
       <c r="G96" s="13" t="s">
         <v>36</v>
@@ -3900,7 +3900,7 @@
         <v>35</v>
       </c>
       <c r="F97" s="12">
-        <v>2195</v>
+        <v>1462</v>
       </c>
       <c r="G97" s="13" t="s">
         <v>36</v>
@@ -3926,7 +3926,7 @@
         <v>35</v>
       </c>
       <c r="F98" s="12">
-        <v>6047</v>
+        <v>2908</v>
       </c>
       <c r="G98" s="13" t="s">
         <v>36</v>
@@ -3952,7 +3952,7 @@
         <v>35</v>
       </c>
       <c r="F99" s="12">
-        <v>8282</v>
+        <v>6279</v>
       </c>
       <c r="G99" s="13" t="s">
         <v>36</v>
@@ -3978,7 +3978,7 @@
         <v>35</v>
       </c>
       <c r="F100" s="12">
-        <v>3287</v>
+        <v>2717</v>
       </c>
       <c r="G100" s="13" t="s">
         <v>36</v>
@@ -4004,7 +4004,7 @@
         <v>35</v>
       </c>
       <c r="F101" s="12">
-        <v>8646</v>
+        <v>4518</v>
       </c>
       <c r="G101" s="13" t="s">
         <v>36</v>
@@ -4030,7 +4030,7 @@
         <v>35</v>
       </c>
       <c r="F102" s="12">
-        <v>2064</v>
+        <v>508</v>
       </c>
       <c r="G102" s="13" t="s">
         <v>36</v>
@@ -4056,7 +4056,7 @@
         <v>35</v>
       </c>
       <c r="F103" s="12">
-        <v>254</v>
+        <v>140</v>
       </c>
       <c r="G103" s="13" t="s">
         <v>36</v>
@@ -4082,7 +4082,7 @@
         <v>35</v>
       </c>
       <c r="F104" s="12">
-        <v>1042</v>
+        <v>442</v>
       </c>
       <c r="G104" s="13" t="s">
         <v>36</v>
@@ -4108,7 +4108,7 @@
         <v>35</v>
       </c>
       <c r="F105" s="12">
-        <v>3775</v>
+        <v>3307</v>
       </c>
       <c r="G105" s="13" t="s">
         <v>36</v>

</xml_diff>